<commit_message>
fix(urdf): declare STL millimetre mesh scale
</commit_message>
<xml_diff>
--- a/03_CAD/URDF/matt_robodog_rev00/reference/Coordinate_Cinematiche_matt_robodog_rev00.xlsx
+++ b/03_CAD/URDF/matt_robodog_rev00/reference/Coordinate_Cinematiche_matt_robodog_rev00.xlsx
@@ -2,17 +2,17 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Joint_Parameters" sheetId="1" r:id="R1aef14a5ec6a4b2d"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Mesh_Transforms" sheetId="2" r:id="R55c82896a21a4ba6"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Reference_Notes" sheetId="3" r:id="Rbf13f7eeb9bc484d"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Link_Engineering" sheetId="4" r:id="R4f9575abea25442e"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Mass_Summary" sheetId="5" r:id="Rbb5f3fdc6baa40a8"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Engineering_Weight_Source" sheetId="6" r:id="R58c9dcc699854f93"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="URDF_Audit" sheetId="7" r:id="R36b9bd6648a0444c"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Inertial_Properties" sheetId="8" r:id="Rc52f2c3cd0764fe5"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="CAD_Source_Data" sheetId="9" r:id="Re29c0b12f341438a"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Mass_Reconciliation" sheetId="10" r:id="Rf788816304f64b13"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Physical_Property_Method" sheetId="11" r:id="Re58eb096c8f14ec6"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Joint_Parameters" sheetId="1" r:id="R17117f0308514131"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Mesh_Transforms" sheetId="2" r:id="R8f9d7fc1e4104cc4"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Reference_Notes" sheetId="3" r:id="R08f3f5507a8d421a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Link_Engineering" sheetId="4" r:id="R1bd136d64b484fc8"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Mass_Summary" sheetId="5" r:id="R01b5bfde62b3429e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Engineering_Weight_Source" sheetId="6" r:id="R47e07315701e4e75"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="URDF_Audit" sheetId="7" r:id="Rf3337a77e49544ce"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Inertial_Properties" sheetId="8" r:id="R50c7af26ae824333"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="CAD_Source_Data" sheetId="9" r:id="R3df41296733f4968"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Mass_Reconciliation" sheetId="10" r:id="R00897d6d28824d0d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Physical_Property_Method" sheetId="11" r:id="Rada7cf4125ca4620"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -319,7 +319,7 @@
   <x:cellStyleXfs count="1">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="393">
+  <x:cellXfs count="405">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
@@ -1316,6 +1316,38 @@
     </x:xf>
     <x:xf numFmtId="0" fontId="19" fillId="28" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="0" applyAlignment="1">
       <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="11" fillId="22" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="11" fillId="22" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="left"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="11" fillId="22" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="left" vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="16" fillId="21" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="16" fillId="21" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="16" fillId="21" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="left" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="16" fillId="21" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="left" vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="11" fillId="22" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="12" fillId="21" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="left" vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="16" fillId="21" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="left" vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="16" fillId="21" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="11" fillId="22" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="left" vertical="center" wrapText="1"/>
     </x:xf>
   </x:cellXfs>
   <x:cellStyles count="1">
@@ -2978,7 +3010,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R2ecf6a50657d4585"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R783632fb57ee4927"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -3484,61 +3516,73 @@
     <x:col min="21" max="21" width="22" hidden="0" customWidth="1"/>
     <x:col min="22" max="22" width="22" hidden="0" customWidth="1"/>
     <x:col min="23" max="23" width="22" hidden="0" customWidth="1"/>
+    <x:col min="24" max="24" width="16" hidden="0" customWidth="1"/>
+    <x:col min="25" max="25" width="18" hidden="0" customWidth="1"/>
+    <x:col min="26" max="26" width="13" hidden="0" customWidth="1"/>
+    <x:col min="27" max="27" width="17" hidden="0" customWidth="1"/>
   </x:cols>
   <x:sheetData>
     <x:row r="1" ht="24" customHeight="1">
-      <x:c r="A1" s="289" t="str">
-        <x:v>MATDOG — Mesh Visual + Collision + proprietà dinamiche</x:v>
-      </x:c>
-      <x:c r="B1" s="289"/>
-      <x:c r="C1" s="289"/>
-      <x:c r="D1" s="289"/>
-      <x:c r="E1" s="289"/>
-      <x:c r="F1" s="289"/>
-      <x:c r="G1" s="289"/>
-      <x:c r="H1" s="289"/>
-      <x:c r="I1" s="289"/>
-      <x:c r="J1" s="289"/>
-      <x:c r="K1" s="289"/>
-      <x:c r="L1" s="289"/>
-      <x:c r="M1" s="289"/>
-      <x:c r="N1" s="289"/>
-      <x:c r="O1" s="289"/>
-      <x:c r="P1" s="289"/>
-      <x:c r="Q1" s="289"/>
-      <x:c r="R1" s="289"/>
-      <x:c r="S1" s="289"/>
-      <x:c r="T1" s="289"/>
-      <x:c r="U1" s="289"/>
-      <x:c r="V1" s="289"/>
-      <x:c r="W1" s="289"/>
+      <x:c r="A1" s="404" t="str">
+        <x:v>MATDOG — Mesh visual + collision + proprietà dinamiche · STL mm → URDF m</x:v>
+      </x:c>
+      <x:c r="B1" s="404"/>
+      <x:c r="C1" s="404"/>
+      <x:c r="D1" s="404"/>
+      <x:c r="E1" s="404"/>
+      <x:c r="F1" s="404"/>
+      <x:c r="G1" s="404"/>
+      <x:c r="H1" s="404"/>
+      <x:c r="I1" s="404"/>
+      <x:c r="J1" s="404"/>
+      <x:c r="K1" s="404"/>
+      <x:c r="L1" s="404"/>
+      <x:c r="M1" s="404"/>
+      <x:c r="N1" s="404"/>
+      <x:c r="O1" s="404"/>
+      <x:c r="P1" s="404"/>
+      <x:c r="Q1" s="404"/>
+      <x:c r="R1" s="404"/>
+      <x:c r="S1" s="404"/>
+      <x:c r="T1" s="404"/>
+      <x:c r="U1" s="404"/>
+      <x:c r="V1" s="404"/>
+      <x:c r="W1" s="404"/>
+      <x:c r="X1" s="156"/>
+      <x:c r="Y1" s="156"/>
+      <x:c r="Z1" s="156"/>
+      <x:c r="AA1" s="156"/>
     </x:row>
     <x:row r="2" ht="36" customHeight="1">
-      <x:c r="A2" s="294" t="str">
-        <x:v>Origini mesh visual/collision: xyz = 0,0,0 m · rpy = 0°,0°,0°. Le colonne di massa e stato inerziale sono aggiornate dal modello CAD dinamico REV00.</x:v>
-      </x:c>
-      <x:c r="B2" s="294"/>
-      <x:c r="C2" s="294"/>
-      <x:c r="D2" s="294"/>
-      <x:c r="E2" s="294"/>
-      <x:c r="F2" s="294"/>
-      <x:c r="G2" s="294"/>
-      <x:c r="H2" s="294"/>
-      <x:c r="I2" s="294"/>
-      <x:c r="J2" s="294"/>
-      <x:c r="K2" s="294"/>
-      <x:c r="L2" s="294"/>
-      <x:c r="M2" s="294"/>
-      <x:c r="N2" s="294"/>
-      <x:c r="O2" s="294"/>
-      <x:c r="P2" s="294"/>
-      <x:c r="Q2" s="294"/>
-      <x:c r="R2" s="294"/>
-      <x:c r="S2" s="294"/>
-      <x:c r="T2" s="294"/>
-      <x:c r="U2" s="294"/>
-      <x:c r="V2" s="294"/>
-      <x:c r="W2" s="294"/>
+      <x:c r="A2" s="399" t="str">
+        <x:v>Origini mesh visual/collision: xyz = 0,0,0 m · rpy = 0°,0°,0°. Gli STL CAD restano in millimetri; ogni &lt;mesh&gt; URDF applica scale="0.001 0.001 0.001".</x:v>
+      </x:c>
+      <x:c r="B2" s="399"/>
+      <x:c r="C2" s="399"/>
+      <x:c r="D2" s="399"/>
+      <x:c r="E2" s="399"/>
+      <x:c r="F2" s="399"/>
+      <x:c r="G2" s="399"/>
+      <x:c r="H2" s="399"/>
+      <x:c r="I2" s="399"/>
+      <x:c r="J2" s="399"/>
+      <x:c r="K2" s="399"/>
+      <x:c r="L2" s="399"/>
+      <x:c r="M2" s="399"/>
+      <x:c r="N2" s="399"/>
+      <x:c r="O2" s="399"/>
+      <x:c r="P2" s="399"/>
+      <x:c r="Q2" s="399"/>
+      <x:c r="R2" s="399"/>
+      <x:c r="S2" s="399"/>
+      <x:c r="T2" s="399"/>
+      <x:c r="U2" s="399"/>
+      <x:c r="V2" s="399"/>
+      <x:c r="W2" s="399"/>
+      <x:c r="X2" s="156"/>
+      <x:c r="Y2" s="156"/>
+      <x:c r="Z2" s="156"/>
+      <x:c r="AA2" s="156"/>
     </x:row>
     <x:row r="5" ht="34" customHeight="1">
       <x:c r="A5" s="345" t="str">
@@ -3624,6 +3668,20 @@
       <x:c r="W5" s="345" t="str">
         <x:v>URDF metadata</x:v>
       </x:c>
+      <x:c r="X5" s="156" t="str">
+        <x:v>Visual scale
+[STL → URDF]</x:v>
+      </x:c>
+      <x:c r="Y5" s="156" t="str">
+        <x:v>Collision scale
+[STL → URDF]</x:v>
+      </x:c>
+      <x:c r="Z5" s="156" t="str">
+        <x:v>STL source unit</x:v>
+      </x:c>
+      <x:c r="AA5" s="156" t="str">
+        <x:v>URDF geometry unit</x:v>
+      </x:c>
     </x:row>
     <x:row r="6" ht="19" customHeight="1">
       <x:c r="A6" s="359" t="str">
@@ -3693,7 +3751,19 @@
         <x:v>URDF &lt;inertial&gt; inserted</x:v>
       </x:c>
       <x:c r="W6" s="301" t="str">
-        <x:v>Simulation-ready</x:v>
+        <x:v>Simulation-ready · mesh scale=0.001</x:v>
+      </x:c>
+      <x:c r="X6" s="156" t="str">
+        <x:v>0.001 0.001 0.001</x:v>
+      </x:c>
+      <x:c r="Y6" s="156" t="str">
+        <x:v>0.001 0.001 0.001</x:v>
+      </x:c>
+      <x:c r="Z6" s="156" t="str">
+        <x:v>mm</x:v>
+      </x:c>
+      <x:c r="AA6" s="156" t="str">
+        <x:v>m</x:v>
       </x:c>
     </x:row>
     <x:row r="7" ht="19" customHeight="1">
@@ -3764,7 +3834,19 @@
         <x:v>URDF &lt;inertial&gt; inserted</x:v>
       </x:c>
       <x:c r="W7" s="301" t="str">
-        <x:v>Simulation-ready</x:v>
+        <x:v>Simulation-ready · mesh scale=0.001</x:v>
+      </x:c>
+      <x:c r="X7" s="156" t="str">
+        <x:v>0.001 0.001 0.001</x:v>
+      </x:c>
+      <x:c r="Y7" s="156" t="str">
+        <x:v>0.001 0.001 0.001</x:v>
+      </x:c>
+      <x:c r="Z7" s="156" t="str">
+        <x:v>mm</x:v>
+      </x:c>
+      <x:c r="AA7" s="156" t="str">
+        <x:v>m</x:v>
       </x:c>
     </x:row>
     <x:row r="8" ht="19" customHeight="1">
@@ -3835,7 +3917,19 @@
         <x:v>URDF &lt;inertial&gt; inserted</x:v>
       </x:c>
       <x:c r="W8" s="301" t="str">
-        <x:v>Simulation-ready</x:v>
+        <x:v>Simulation-ready · mesh scale=0.001</x:v>
+      </x:c>
+      <x:c r="X8" s="156" t="str">
+        <x:v>0.001 0.001 0.001</x:v>
+      </x:c>
+      <x:c r="Y8" s="156" t="str">
+        <x:v>0.001 0.001 0.001</x:v>
+      </x:c>
+      <x:c r="Z8" s="156" t="str">
+        <x:v>mm</x:v>
+      </x:c>
+      <x:c r="AA8" s="156" t="str">
+        <x:v>m</x:v>
       </x:c>
     </x:row>
     <x:row r="9" ht="19" customHeight="1">
@@ -3906,7 +4000,19 @@
         <x:v>URDF &lt;inertial&gt; inserted</x:v>
       </x:c>
       <x:c r="W9" s="301" t="str">
-        <x:v>Simulation-ready</x:v>
+        <x:v>Simulation-ready · mesh scale=0.001</x:v>
+      </x:c>
+      <x:c r="X9" s="156" t="str">
+        <x:v>0.001 0.001 0.001</x:v>
+      </x:c>
+      <x:c r="Y9" s="156" t="str">
+        <x:v>0.001 0.001 0.001</x:v>
+      </x:c>
+      <x:c r="Z9" s="156" t="str">
+        <x:v>mm</x:v>
+      </x:c>
+      <x:c r="AA9" s="156" t="str">
+        <x:v>m</x:v>
       </x:c>
     </x:row>
     <x:row r="10" ht="19" customHeight="1">
@@ -3977,7 +4083,19 @@
         <x:v>URDF &lt;inertial&gt; inserted</x:v>
       </x:c>
       <x:c r="W10" s="301" t="str">
-        <x:v>Simulation-ready</x:v>
+        <x:v>Simulation-ready · mesh scale=0.001</x:v>
+      </x:c>
+      <x:c r="X10" s="156" t="str">
+        <x:v>0.001 0.001 0.001</x:v>
+      </x:c>
+      <x:c r="Y10" s="156" t="str">
+        <x:v>0.001 0.001 0.001</x:v>
+      </x:c>
+      <x:c r="Z10" s="156" t="str">
+        <x:v>mm</x:v>
+      </x:c>
+      <x:c r="AA10" s="156" t="str">
+        <x:v>m</x:v>
       </x:c>
     </x:row>
     <x:row r="11" ht="19" customHeight="1">
@@ -4048,7 +4166,19 @@
         <x:v>URDF &lt;inertial&gt; inserted</x:v>
       </x:c>
       <x:c r="W11" s="301" t="str">
-        <x:v>Simulation-ready</x:v>
+        <x:v>Simulation-ready · mesh scale=0.001</x:v>
+      </x:c>
+      <x:c r="X11" s="156" t="str">
+        <x:v>0.001 0.001 0.001</x:v>
+      </x:c>
+      <x:c r="Y11" s="156" t="str">
+        <x:v>0.001 0.001 0.001</x:v>
+      </x:c>
+      <x:c r="Z11" s="156" t="str">
+        <x:v>mm</x:v>
+      </x:c>
+      <x:c r="AA11" s="156" t="str">
+        <x:v>m</x:v>
       </x:c>
     </x:row>
     <x:row r="12" ht="19" customHeight="1">
@@ -4119,7 +4249,19 @@
         <x:v>URDF &lt;inertial&gt; inserted</x:v>
       </x:c>
       <x:c r="W12" s="301" t="str">
-        <x:v>Simulation-ready</x:v>
+        <x:v>Simulation-ready · mesh scale=0.001</x:v>
+      </x:c>
+      <x:c r="X12" s="156" t="str">
+        <x:v>0.001 0.001 0.001</x:v>
+      </x:c>
+      <x:c r="Y12" s="156" t="str">
+        <x:v>0.001 0.001 0.001</x:v>
+      </x:c>
+      <x:c r="Z12" s="156" t="str">
+        <x:v>mm</x:v>
+      </x:c>
+      <x:c r="AA12" s="156" t="str">
+        <x:v>m</x:v>
       </x:c>
     </x:row>
     <x:row r="13" ht="19" customHeight="1">
@@ -4190,7 +4332,19 @@
         <x:v>URDF &lt;inertial&gt; inserted</x:v>
       </x:c>
       <x:c r="W13" s="301" t="str">
-        <x:v>Simulation-ready</x:v>
+        <x:v>Simulation-ready · mesh scale=0.001</x:v>
+      </x:c>
+      <x:c r="X13" s="156" t="str">
+        <x:v>0.001 0.001 0.001</x:v>
+      </x:c>
+      <x:c r="Y13" s="156" t="str">
+        <x:v>0.001 0.001 0.001</x:v>
+      </x:c>
+      <x:c r="Z13" s="156" t="str">
+        <x:v>mm</x:v>
+      </x:c>
+      <x:c r="AA13" s="156" t="str">
+        <x:v>m</x:v>
       </x:c>
     </x:row>
     <x:row r="14" ht="19" customHeight="1">
@@ -4261,7 +4415,19 @@
         <x:v>URDF &lt;inertial&gt; inserted</x:v>
       </x:c>
       <x:c r="W14" s="301" t="str">
-        <x:v>Simulation-ready</x:v>
+        <x:v>Simulation-ready · mesh scale=0.001</x:v>
+      </x:c>
+      <x:c r="X14" s="156" t="str">
+        <x:v>0.001 0.001 0.001</x:v>
+      </x:c>
+      <x:c r="Y14" s="156" t="str">
+        <x:v>0.001 0.001 0.001</x:v>
+      </x:c>
+      <x:c r="Z14" s="156" t="str">
+        <x:v>mm</x:v>
+      </x:c>
+      <x:c r="AA14" s="156" t="str">
+        <x:v>m</x:v>
       </x:c>
     </x:row>
     <x:row r="15" ht="19" customHeight="1">
@@ -4332,7 +4498,19 @@
         <x:v>URDF &lt;inertial&gt; inserted</x:v>
       </x:c>
       <x:c r="W15" s="301" t="str">
-        <x:v>Simulation-ready</x:v>
+        <x:v>Simulation-ready · mesh scale=0.001</x:v>
+      </x:c>
+      <x:c r="X15" s="156" t="str">
+        <x:v>0.001 0.001 0.001</x:v>
+      </x:c>
+      <x:c r="Y15" s="156" t="str">
+        <x:v>0.001 0.001 0.001</x:v>
+      </x:c>
+      <x:c r="Z15" s="156" t="str">
+        <x:v>mm</x:v>
+      </x:c>
+      <x:c r="AA15" s="156" t="str">
+        <x:v>m</x:v>
       </x:c>
     </x:row>
     <x:row r="16" ht="19" customHeight="1">
@@ -4403,7 +4581,19 @@
         <x:v>URDF &lt;inertial&gt; inserted</x:v>
       </x:c>
       <x:c r="W16" s="301" t="str">
-        <x:v>Simulation-ready</x:v>
+        <x:v>Simulation-ready · mesh scale=0.001</x:v>
+      </x:c>
+      <x:c r="X16" s="156" t="str">
+        <x:v>0.001 0.001 0.001</x:v>
+      </x:c>
+      <x:c r="Y16" s="156" t="str">
+        <x:v>0.001 0.001 0.001</x:v>
+      </x:c>
+      <x:c r="Z16" s="156" t="str">
+        <x:v>mm</x:v>
+      </x:c>
+      <x:c r="AA16" s="156" t="str">
+        <x:v>m</x:v>
       </x:c>
     </x:row>
     <x:row r="17" ht="19" customHeight="1">
@@ -4474,7 +4664,19 @@
         <x:v>URDF &lt;inertial&gt; inserted</x:v>
       </x:c>
       <x:c r="W17" s="301" t="str">
-        <x:v>Simulation-ready</x:v>
+        <x:v>Simulation-ready · mesh scale=0.001</x:v>
+      </x:c>
+      <x:c r="X17" s="156" t="str">
+        <x:v>0.001 0.001 0.001</x:v>
+      </x:c>
+      <x:c r="Y17" s="156" t="str">
+        <x:v>0.001 0.001 0.001</x:v>
+      </x:c>
+      <x:c r="Z17" s="156" t="str">
+        <x:v>mm</x:v>
+      </x:c>
+      <x:c r="AA17" s="156" t="str">
+        <x:v>m</x:v>
       </x:c>
     </x:row>
     <x:row r="18" ht="19" customHeight="1">
@@ -4545,7 +4747,19 @@
         <x:v>URDF &lt;inertial&gt; inserted</x:v>
       </x:c>
       <x:c r="W18" s="301" t="str">
-        <x:v>Simulation-ready</x:v>
+        <x:v>Simulation-ready · mesh scale=0.001</x:v>
+      </x:c>
+      <x:c r="X18" s="156" t="str">
+        <x:v>0.001 0.001 0.001</x:v>
+      </x:c>
+      <x:c r="Y18" s="156" t="str">
+        <x:v>0.001 0.001 0.001</x:v>
+      </x:c>
+      <x:c r="Z18" s="156" t="str">
+        <x:v>mm</x:v>
+      </x:c>
+      <x:c r="AA18" s="156" t="str">
+        <x:v>m</x:v>
       </x:c>
     </x:row>
     <x:row r="19" ht="19" customHeight="1">
@@ -4616,7 +4830,19 @@
         <x:v>URDF &lt;inertial&gt; inserted</x:v>
       </x:c>
       <x:c r="W19" s="301" t="str">
-        <x:v>Simulation-ready</x:v>
+        <x:v>Simulation-ready · mesh scale=0.001</x:v>
+      </x:c>
+      <x:c r="X19" s="156" t="str">
+        <x:v>0.001 0.001 0.001</x:v>
+      </x:c>
+      <x:c r="Y19" s="156" t="str">
+        <x:v>0.001 0.001 0.001</x:v>
+      </x:c>
+      <x:c r="Z19" s="156" t="str">
+        <x:v>mm</x:v>
+      </x:c>
+      <x:c r="AA19" s="156" t="str">
+        <x:v>m</x:v>
       </x:c>
     </x:row>
     <x:row r="20" ht="19" customHeight="1">
@@ -4687,7 +4913,19 @@
         <x:v>URDF &lt;inertial&gt; inserted</x:v>
       </x:c>
       <x:c r="W20" s="301" t="str">
-        <x:v>Simulation-ready</x:v>
+        <x:v>Simulation-ready · mesh scale=0.001</x:v>
+      </x:c>
+      <x:c r="X20" s="156" t="str">
+        <x:v>0.001 0.001 0.001</x:v>
+      </x:c>
+      <x:c r="Y20" s="156" t="str">
+        <x:v>0.001 0.001 0.001</x:v>
+      </x:c>
+      <x:c r="Z20" s="156" t="str">
+        <x:v>mm</x:v>
+      </x:c>
+      <x:c r="AA20" s="156" t="str">
+        <x:v>m</x:v>
       </x:c>
     </x:row>
     <x:row r="21" ht="19" customHeight="1">
@@ -4758,7 +4996,19 @@
         <x:v>URDF &lt;inertial&gt; inserted</x:v>
       </x:c>
       <x:c r="W21" s="301" t="str">
-        <x:v>Simulation-ready</x:v>
+        <x:v>Simulation-ready · mesh scale=0.001</x:v>
+      </x:c>
+      <x:c r="X21" s="156" t="str">
+        <x:v>0.001 0.001 0.001</x:v>
+      </x:c>
+      <x:c r="Y21" s="156" t="str">
+        <x:v>0.001 0.001 0.001</x:v>
+      </x:c>
+      <x:c r="Z21" s="156" t="str">
+        <x:v>mm</x:v>
+      </x:c>
+      <x:c r="AA21" s="156" t="str">
+        <x:v>m</x:v>
       </x:c>
     </x:row>
     <x:row r="22" ht="19" customHeight="1">
@@ -4829,7 +5079,19 @@
         <x:v>URDF &lt;inertial&gt; inserted</x:v>
       </x:c>
       <x:c r="W22" s="301" t="str">
-        <x:v>Simulation-ready</x:v>
+        <x:v>Simulation-ready · mesh scale=0.001</x:v>
+      </x:c>
+      <x:c r="X22" s="156" t="str">
+        <x:v>0.001 0.001 0.001</x:v>
+      </x:c>
+      <x:c r="Y22" s="156" t="str">
+        <x:v>0.001 0.001 0.001</x:v>
+      </x:c>
+      <x:c r="Z22" s="156" t="str">
+        <x:v>mm</x:v>
+      </x:c>
+      <x:c r="AA22" s="156" t="str">
+        <x:v>m</x:v>
       </x:c>
     </x:row>
     <x:row r="24">
@@ -4892,7 +5154,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R94ad51e75eba4da9"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rdb06a6cc5bb6411d"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -4944,16 +5206,18 @@
         <x:v>File URDF finale</x:v>
       </x:c>
       <x:c r="B5" s="43" t="str">
-        <x:v>matt_robodog_rev00_final_kinematics_mass_material_lowerlimit92_clean.urdf</x:v>
-      </x:c>
+        <x:v>matt_robodog_rev00.urdf</x:v>
+      </x:c>
+      <x:c r="C5"/>
     </x:row>
     <x:row r="6">
       <x:c r="A6" s="90" t="str">
         <x:v>Stato</x:v>
       </x:c>
       <x:c r="B6" s="95" t="str">
-        <x:v>Baseline cinematica approvata</x:v>
-      </x:c>
+        <x:v>Baseline cinematica + dinamica + scala mesh approvata</x:v>
+      </x:c>
+      <x:c r="C6"/>
     </x:row>
     <x:row r="8">
       <x:c r="A8" s="100" t="str">
@@ -5062,6 +5326,17 @@
       <x:c r="F14" s="115"/>
       <x:c r="G14" s="115"/>
       <x:c r="H14" s="115"/>
+    </x:row>
+    <x:row r="15">
+      <x:c r="A15" t="str">
+        <x:v>7</x:v>
+      </x:c>
+      <x:c r="B15" t="str">
+        <x:v>Unità mesh STL</x:v>
+      </x:c>
+      <x:c r="C15" s="156" t="str">
+        <x:v>Vertici STL esportati dal CAD in mm. In ogni mesh visual e collision URDF: scale="0.001 0.001 0.001"; joint, CoM e inerzie restano in unità SI.</x:v>
+      </x:c>
     </x:row>
     <x:row r="16">
       <x:c r="A16" s="121" t="str">
@@ -5923,7 +6198,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R019e2d942cee4562"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R4e033e6dd49543d3"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -7413,7 +7688,7 @@
     </x:row>
     <x:row r="2" ht="34" customHeight="1">
       <x:c r="A2" s="294" t="str">
-        <x:v>Audit aggiornato: struttura, riferimenti mesh, origini visual/collision, limiti, masse CAD, CoM per-link e tensori d’inerzia.</x:v>
+        <x:v>Audit aggiornato: struttura, joint, mesh, scala STL mm→m, limiti, masse CAD, CoM per-link e tensori d’inerzia.</x:v>
       </x:c>
       <x:c r="B2" s="294"/>
       <x:c r="C2" s="294"/>
@@ -7530,13 +7805,13 @@
         <x:v>PASS</x:v>
       </x:c>
       <x:c r="C10" s="301" t="str">
-        <x:v>34 riferimenti mesh (visual + collision), tutti relativi a meshes/*.stl; 17 asset unici.</x:v>
+        <x:v>34 riferimenti mesh (visual + collision), tutti relativi a meshes/*.stl; 17 asset unici; ogni mesh dichiara scale="0.001 0.001 0.001".</x:v>
       </x:c>
       <x:c r="D10" s="301" t="str">
-        <x:v>Nessuna.</x:v>
+        <x:v>Scala URDF dichiarata per STL CAD in mm.</x:v>
       </x:c>
       <x:c r="E10" s="301" t="str">
-        <x:v>Pulito</x:v>
+        <x:v>Canonico</x:v>
       </x:c>
     </x:row>
     <x:row r="11" ht="38" customHeight="1">

</xml_diff>